<commit_message>
v11 legacy transgenes + clutch labels + overview pages
</commit_message>
<xml_diff>
--- a/seed_kits/legacy_wrangling_v2/raw/Unique_parent_names__mom_dad_combined__preview_dqm.xlsx
+++ b/seed_kits/legacy_wrangling_v2/raw/Unique_parent_names__mom_dad_combined__preview_dqm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/legacy_wrangling_v2/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62EEDAB-44BF-0C45-A7F1-E7DCEA3656CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6D53B4-29E3-7247-9AAD-30AF03E8B2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="2900" windowWidth="34560" windowHeight="19860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="19860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - Unique_parent_names__" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="81">
   <si>
     <t>parent_fish_name</t>
   </si>
@@ -199,9 +199,6 @@
     <t>pSWIN04</t>
   </si>
   <si>
-    <t>pSWIN05</t>
-  </si>
-  <si>
     <t>is01</t>
   </si>
   <si>
@@ -212,9 +209,6 @@
   </si>
   <si>
     <t>is04</t>
-  </si>
-  <si>
-    <t>is05</t>
   </si>
   <si>
     <t>injected_rna</t>
@@ -310,7 +304,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -322,7 +316,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1477,174 +1470,189 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2">
-        <v>301</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2">
-        <v>302</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2">
-        <v>315</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="C6" s="2">
-        <v>325</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2">
-        <v>315</v>
+        <v>302</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2">
-        <v>315</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>60</v>
+        <v>41</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2">
+        <v>305</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="2">
-        <v>301</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
+      <c r="A12" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>4</v>
+      </c>
+      <c r="C12" s="2">
+        <v>301</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="2">
-        <v>302</v>
+        <v>301</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="2" t="s">
-        <v>19</v>
+      <c r="A14" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2">
+        <v>301</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="2">
-        <v>318</v>
+        <v>68</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2">
-        <v>316</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>29</v>
@@ -1655,139 +1663,139 @@
     </row>
     <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C19" s="2">
-        <v>321</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2">
-        <v>336</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2">
-        <v>301</v>
+        <v>317</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="2">
-        <v>310</v>
+      <c r="A22" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="3">
+        <v>309</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="2">
-        <v>310</v>
+        <v>71</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="3">
+        <v>309</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>7</v>
+        <v>45</v>
+      </c>
+      <c r="C24" s="2">
+        <v>318</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C25" s="2">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="C26" s="2">
-        <v>325</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>63</v>
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="2">
+        <v>320</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>64</v>
+        <v>24</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="2">
+        <v>321</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="C29" s="2">
-        <v>325</v>
+        <v>314</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>9</v>
@@ -1798,246 +1806,234 @@
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C31" s="2">
-        <v>325</v>
+        <v>315</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C32" s="2">
-        <v>305</v>
+        <v>315</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C33" s="2">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C34" s="2">
-        <v>327</v>
+        <v>315</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>45</v>
+      <c r="A35" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="C35" s="2">
-        <v>318</v>
+        <v>315</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>29</v>
+      <c r="A36" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="C36" s="2">
-        <v>309</v>
+        <v>315</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C37" s="2">
-        <v>314</v>
+        <v>32</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C38" s="2">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C39" s="2">
-        <v>304</v>
+        <v>325</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C40" s="2">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>4</v>
+      <c r="A41" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="C41" s="2">
-        <v>301</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>66</v>
+        <v>325</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>4</v>
+        <v>40</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="C42" s="2">
-        <v>301</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>66</v>
+        <v>325</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="5" t="s">
-        <v>68</v>
+      <c r="A43" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C43" s="2">
-        <v>315</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>69</v>
+        <v>327</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C44" s="2">
+        <v>325</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A45" s="3" t="s">
-        <v>82</v>
+      <c r="A45" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C45" s="3">
-        <v>309</v>
+        <v>55</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A46" s="5" t="s">
-        <v>73</v>
+      <c r="A46" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C46" s="3">
-        <v>309</v>
+        <v>56</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A47" s="6" t="s">
-        <v>75</v>
+      <c r="A47" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="2">
-        <v>301</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>69</v>
+        <v>57</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A48" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C48" s="2">
-        <v>315</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A49" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C49" s="2">
-        <v>325</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A50" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50" s="2">
-        <v>315</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>81</v>
+      <c r="A48" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A49" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A50" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E50">
+    <sortCondition ref="B1:B50"/>
+  </sortState>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
   <headerFooter>

</xml_diff>